<commit_message>
Boekhouding: Q4-pakket t/m 26/10, bpost-koppeling, btw lopend
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFdhoSd4GqAxUvFp4Qt
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
@@ -467,7 +467,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-26)</t>
+          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2172.18</v>
+        <v>2163.58</v>
       </c>
     </row>
     <row r="6">
@@ -1135,7 +1135,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Leningen en rekening-courant op 2026-10-26 (uit de bank)</t>
+          <t>Leningen en rekening-courant op 2026-10-27 (uit de bank)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ochtendcheck 28/10: Q4-pakket, btw lopend, rapporten
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFbbPRuSBDVoyyn4ADA
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
@@ -467,7 +467,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-27)</t>
+          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-28)</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Leningen en rekening-courant op 2026-10-27 (uit de bank)</t>
+          <t>Leningen en rekening-courant op 2026-10-28 (uit de bank)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ochtendcheck 30/10: boekhoudrapporten en lopende btw bijgewerkt
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFch5kQj8jLjKJq7ZAQ
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Jaarafsluiting_2026.xlsx
@@ -467,7 +467,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-28)</t>
+          <t>SmartPaw VOF — jaarafsluiting 2026 (voorbereiding voor Pro-count, stand 2026-10-30)</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-1024.72</v>
+        <v>2169.16</v>
       </c>
     </row>
     <row r="6">
@@ -1135,7 +1135,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Leningen en rekening-courant op 2026-10-28 (uit de bank)</t>
+          <t>Leningen en rekening-courant op 2026-10-30 (uit de bank)</t>
         </is>
       </c>
     </row>

</xml_diff>